<commit_message>
work in progress. Changed wright species not current panama woody
</commit_message>
<xml_diff>
--- a/splists_out/needs_revision/plotsbci_not_garwood.xlsx
+++ b/splists_out/needs_revision/plotsbci_not_garwood.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AY6"/>
+  <dimension ref="A1:AU6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -447,167 +447,147 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>forestgeo_current_name</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>orig_infraspecies_rank</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>sp6prior</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>IDLevel</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_matched_name</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_matched_authors</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_matched_rank</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_matched_status</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_matched_plant_name_id</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_matched_ipni_id</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>match_similarity</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_accepted_plant_name_id</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_accepted_powo_id</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_accepted_ipni_id</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_accepted_binomial</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_accepted_name</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_accepted_authority</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_accepted_family</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_accepted_genus</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_accepted_species</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_accepted_infrarank</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_accepted_infraspecies</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_accepted_rank</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_accepted_lifeform</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>origmatches</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>names_notes</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>wcvp_accepted_duplicated</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>sp4</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
           <t>orig_name</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>orig_infraspecies_rank</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>sp6prior</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>IDLevel</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_matched_name</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_matched_authors</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_matched_rank</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_matched_status</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_matched_plant_name_id</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_matched_ipni_id</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>match_similarity</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_accepted_plant_name_id</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_accepted_powo_id</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_accepted_ipni_id</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_accepted_binomial</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_accepted_name</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_accepted_authority</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_accepted_family</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_accepted_genus</t>
-        </is>
-      </c>
-      <c r="AL1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_accepted_species</t>
-        </is>
-      </c>
-      <c r="AM1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_accepted_infrarank</t>
-        </is>
-      </c>
-      <c r="AN1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_accepted_infraspecies</t>
-        </is>
-      </c>
-      <c r="AO1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_accepted_rank</t>
-        </is>
-      </c>
-      <c r="AP1" s="1" t="inlineStr">
-        <is>
-          <t>wcvp_accepted_lifeform</t>
-        </is>
-      </c>
-      <c r="AQ1" s="1" t="inlineStr">
-        <is>
-          <t>origmatches</t>
-        </is>
-      </c>
-      <c r="AR1" s="1" t="inlineStr">
-        <is>
-          <t>names_notes</t>
-        </is>
-      </c>
-      <c r="AS1" s="1" t="inlineStr">
-        <is>
-          <t>current_name</t>
-        </is>
-      </c>
-      <c r="AT1" s="1" t="inlineStr">
-        <is>
-          <t>current_authority</t>
-        </is>
-      </c>
-      <c r="AU1" s="1" t="inlineStr">
-        <is>
-          <t>current_family</t>
-        </is>
-      </c>
-      <c r="AV1" s="1" t="inlineStr">
-        <is>
-          <t>current_genus</t>
-        </is>
-      </c>
-      <c r="AW1" s="1" t="inlineStr">
-        <is>
-          <t>current_species</t>
-        </is>
-      </c>
-      <c r="AX1" s="1" t="inlineStr">
-        <is>
-          <t>current_binomial</t>
-        </is>
-      </c>
-      <c r="AY1" s="1" t="inlineStr">
-        <is>
-          <t>sp4</t>
         </is>
       </c>
     </row>
@@ -787,6 +767,16 @@
           <t>TRUE</t>
         </is>
       </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>Jupunba idiopoda</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -964,9 +954,19 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AY3" t="inlineStr">
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AT3" t="inlineStr">
         <is>
           <t>CUP2</t>
+        </is>
+      </c>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>Cupania scrobiculata</t>
         </is>
       </c>
     </row>
@@ -1146,9 +1146,19 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AY4" t="inlineStr">
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AT4" t="inlineStr">
         <is>
           <t>MYRF</t>
+        </is>
+      </c>
+      <c r="AU4" t="inlineStr">
+        <is>
+          <t>Myrciaria floribunda</t>
         </is>
       </c>
     </row>
@@ -1328,9 +1338,19 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AY5" t="inlineStr">
+      <c r="AS5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AT5" t="inlineStr">
         <is>
           <t>NEC2</t>
+        </is>
+      </c>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>Nectandra cuspidata</t>
         </is>
       </c>
     </row>
@@ -1510,9 +1530,19 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AY6" t="inlineStr">
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr">
         <is>
           <t>UNO2</t>
+        </is>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>Unonopsis panamensis</t>
         </is>
       </c>
     </row>

</xml_diff>